<commit_message>
Implementar sincronização automática de vendas do Nuvemshop
</commit_message>
<xml_diff>
--- a/VENDAS.xlsx
+++ b/VENDAS.xlsx
@@ -1,31 +1,31 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" tabRatio="617" firstSheet="9" activeTab="19" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="JAN" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="FEV" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="MAR" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="ABR" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="MAIO" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="JUN" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="JULH" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="AGOS" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="SET" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="OUT" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="NOV" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="GERAL" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet name="2020" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet name="2021" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet name="2022" sheetId="15" state="visible" r:id="rId15"/>
-    <sheet name="2023" sheetId="16" state="visible" r:id="rId16"/>
-    <sheet name="2024" sheetId="17" state="visible" r:id="rId17"/>
-    <sheet name="2025" sheetId="18" state="visible" r:id="rId18"/>
-    <sheet name="2026" sheetId="19" state="visible" r:id="rId19"/>
-    <sheet name="GRAFICO 5 ANOS" sheetId="20" state="visible" r:id="rId20"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="JAN" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FEV" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MAR" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ABR" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MAIO" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="JUN" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="JULH" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AGOS" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SET" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="OUT" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="NOV" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="GERAL" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2020" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2021" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2022" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2023" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2024" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2025" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2026" sheetId="19" state="visible" r:id="rId19"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="GRAFICO 5 ANOS" sheetId="20" state="visible" r:id="rId20"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
@@ -1599,7 +1599,7 @@
 </file>
 
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <plotArea>
       <layout>
@@ -1633,7 +1633,7 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln w="22225" cap="rnd">
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="22225" cap="rnd">
               <a:solidFill>
                 <a:schemeClr val="accent1"/>
               </a:solidFill>
@@ -1643,25 +1643,25 @@
           <marker>
             <symbol val="none"/>
             <spPr>
-              <a:ln>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
           </marker>
           <dLbls>
             <spPr>
-              <a:noFill/>
-              <a:ln>
+              <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
             <txPr>
-              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
                 <a:spAutoFit/>
               </a:bodyPr>
-              <a:lstStyle/>
-              <a:p>
+              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr sz="1200" b="0" i="0" strike="noStrike" kern="1200" baseline="0">
                     <a:solidFill>
@@ -1849,7 +1849,7 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln w="22225" cap="rnd">
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="22225" cap="rnd">
               <a:solidFill>
                 <a:schemeClr val="accent2"/>
               </a:solidFill>
@@ -1859,7 +1859,7 @@
           <marker>
             <symbol val="none"/>
             <spPr>
-              <a:ln>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
@@ -1876,18 +1876,18 @@
               <showBubbleSize val="0"/>
             </dLbl>
             <spPr>
-              <a:noFill/>
-              <a:ln>
+              <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
             <txPr>
-              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
                 <a:spAutoFit/>
               </a:bodyPr>
-              <a:lstStyle/>
-              <a:p>
+              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr sz="1200" b="0" i="0" strike="noStrike" kern="1200" baseline="0">
                     <a:solidFill>
@@ -2075,7 +2075,7 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln w="22225" cap="rnd">
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="22225" cap="rnd">
               <a:solidFill>
                 <a:schemeClr val="accent3"/>
               </a:solidFill>
@@ -2085,7 +2085,7 @@
           <marker>
             <symbol val="none"/>
             <spPr>
-              <a:ln>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
@@ -2102,18 +2102,18 @@
               <showBubbleSize val="0"/>
             </dLbl>
             <spPr>
-              <a:noFill/>
-              <a:ln>
+              <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
             <txPr>
-              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
                 <a:spAutoFit/>
               </a:bodyPr>
-              <a:lstStyle/>
-              <a:p>
+              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr sz="1200" b="0" i="0" strike="noStrike" kern="1200" baseline="0">
                     <a:solidFill>
@@ -2316,16 +2316,16 @@
         <minorTickMark val="none"/>
         <tickLblPos val="nextTo"/>
         <spPr>
-          <a:noFill/>
-          <a:ln>
+          <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:noFill/>
             <a:prstDash val="solid"/>
           </a:ln>
         </spPr>
         <txPr>
-          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-          <a:lstStyle/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr sz="900" b="0" i="0" strike="noStrike" kern="1200" baseline="0">
                 <a:solidFill>
@@ -2383,16 +2383,16 @@
       </layout>
       <overlay val="0"/>
       <spPr>
-        <a:noFill/>
-        <a:ln>
+        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
       </spPr>
       <txPr>
-        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-        <a:lstStyle/>
-        <a:p>
+        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:pPr>
             <a:defRPr sz="900" b="0" i="0" strike="noStrike" kern="1200" baseline="0">
               <a:solidFill>
@@ -2416,13 +2416,13 @@
     <dispBlanksAs val="gap"/>
   </chart>
   <spPr>
-    <a:solidFill>
+    <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
       <a:schemeClr val="dk1">
         <a:lumMod val="75000"/>
         <a:lumOff val="25000"/>
       </a:schemeClr>
     </a:solidFill>
-    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+    <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9525" cap="flat" cmpd="sng" algn="ctr">
       <a:solidFill>
         <a:schemeClr val="dk1">
           <a:lumMod val="15000"/>
@@ -2437,7 +2437,7 @@
 </file>
 
 <file path=xl/charts/chart10.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <plotArea>
       <layout>
@@ -2472,7 +2472,7 @@
             </strRef>
           </tx>
           <spPr>
-            <a:gradFill rotWithShape="1">
+            <a:gradFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rotWithShape="1">
               <a:gsLst>
                 <a:gs pos="0">
                   <a:schemeClr val="accent1">
@@ -2495,7 +2495,7 @@
               </a:gsLst>
               <a:lin ang="16200000" scaled="0"/>
             </a:gradFill>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -2507,7 +2507,7 @@
                 <rot lat="0" lon="0" rev="1200000"/>
               </lightRig>
             </scene3d>
-            <a:sp3d>
+            <a:sp3d xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <bevelT w="63500" h="25400"/>
             </a:sp3d>
           </spPr>
@@ -2546,18 +2546,18 @@
             <dLbl>
               <idx val="8"/>
               <spPr>
-                <a:noFill/>
-                <a:ln>
+                <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:noFill/>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
                   <a:noAutofit/>
                 </a:bodyPr>
-                <a:lstStyle/>
-                <a:p>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="1100" b="0" i="0" strike="noStrike" kern="1200" baseline="0">
                       <a:solidFill>
@@ -2605,18 +2605,18 @@
               <showBubbleSize val="0"/>
             </dLbl>
             <spPr>
-              <a:noFill/>
-              <a:ln>
+              <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
             <txPr>
-              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
                 <a:spAutoFit/>
               </a:bodyPr>
-              <a:lstStyle/>
-              <a:p>
+              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr sz="1100" b="0" i="0" strike="noStrike" kern="1200" baseline="0">
                     <a:solidFill>
@@ -2749,10 +2749,10 @@
             </strRef>
           </tx>
           <spPr>
-            <a:solidFill>
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:srgbClr val="00FF00"/>
             </a:solidFill>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -2764,7 +2764,7 @@
                 <rot lat="0" lon="0" rev="1200000"/>
               </lightRig>
             </scene3d>
-            <a:sp3d>
+            <a:sp3d xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <bevelT w="63500" h="25400"/>
             </a:sp3d>
           </spPr>
@@ -2803,18 +2803,18 @@
             <dLbl>
               <idx val="8"/>
               <spPr>
-                <a:noFill/>
-                <a:ln>
+                <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:noFill/>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
                   <a:noAutofit/>
                 </a:bodyPr>
-                <a:lstStyle/>
-                <a:p>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" i="0" strike="noStrike" kern="1200" baseline="0">
                       <a:solidFill>
@@ -2852,18 +2852,18 @@
               <showBubbleSize val="0"/>
             </dLbl>
             <spPr>
-              <a:noFill/>
-              <a:ln>
+              <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
             <txPr>
-              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
                 <a:spAutoFit/>
               </a:bodyPr>
-              <a:lstStyle/>
-              <a:p>
+              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr sz="1000" b="0" i="0" strike="noStrike" kern="1200" baseline="0">
                     <a:solidFill>
@@ -2996,10 +2996,10 @@
             </strRef>
           </tx>
           <spPr>
-            <a:solidFill>
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:srgbClr val="FF0000"/>
             </a:solidFill>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -3011,7 +3011,7 @@
                 <rot lat="0" lon="0" rev="1200000"/>
               </lightRig>
             </scene3d>
-            <a:sp3d>
+            <a:sp3d xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <bevelT w="63500" h="25400"/>
             </a:sp3d>
           </spPr>
@@ -3028,18 +3028,18 @@
               <showBubbleSize val="0"/>
             </dLbl>
             <spPr>
-              <a:noFill/>
-              <a:ln>
+              <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
             <txPr>
-              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
                 <a:spAutoFit/>
               </a:bodyPr>
-              <a:lstStyle/>
-              <a:p>
+              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr sz="900" b="0" i="0" strike="noStrike" kern="1200" baseline="0">
                     <a:solidFill>
@@ -3183,8 +3183,8 @@
         <minorTickMark val="none"/>
         <tickLblPos val="nextTo"/>
         <spPr>
-          <a:noFill/>
-          <a:ln w="12700" cap="flat" cmpd="sng" algn="ctr">
+          <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12700" cap="flat" cmpd="sng" algn="ctr">
             <a:solidFill>
               <a:schemeClr val="lt1">
                 <a:alpha val="54000"/>
@@ -3196,9 +3196,9 @@
           </a:ln>
         </spPr>
         <txPr>
-          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-          <a:lstStyle/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr sz="900" b="0" i="0" strike="noStrike" kern="1200" baseline="0">
                 <a:solidFill>
@@ -3244,16 +3244,16 @@
       <legendPos val="b"/>
       <overlay val="0"/>
       <spPr>
-        <a:noFill/>
-        <a:ln>
+        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
       </spPr>
       <txPr>
-        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-        <a:lstStyle/>
-        <a:p>
+        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:pPr>
             <a:defRPr sz="900" b="0" i="0" strike="noStrike" kern="1200" baseline="0">
               <a:solidFill>
@@ -3277,7 +3277,7 @@
     <dispBlanksAs val="gap"/>
   </chart>
   <spPr>
-    <a:gradFill rotWithShape="1">
+    <a:gradFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rotWithShape="1">
       <a:gsLst>
         <a:gs pos="0">
           <a:schemeClr val="dk1">
@@ -3297,7 +3297,7 @@
       </a:path>
       <a:tileRect/>
     </a:gradFill>
-    <a:ln>
+    <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
       <a:noFill/>
       <a:prstDash val="solid"/>
     </a:ln>
@@ -3306,13 +3306,13 @@
 </file>
 
 <file path=xl/charts/chart11.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:r>
               <a:t>None</a:t>
             </a:r>
@@ -3342,7 +3342,7 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
@@ -3483,7 +3483,7 @@
 </file>
 
 <file path=xl/charts/chart12.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <plotArea>
       <layout>
@@ -3518,7 +3518,7 @@
             </strRef>
           </tx>
           <spPr>
-            <a:gradFill rotWithShape="1">
+            <a:gradFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rotWithShape="1">
               <a:gsLst>
                 <a:gs pos="0">
                   <a:schemeClr val="accent1">
@@ -3541,7 +3541,7 @@
               </a:gsLst>
               <a:lin ang="16200000" scaled="0"/>
             </a:gradFill>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -3553,7 +3553,7 @@
                 <rot lat="0" lon="0" rev="1200000"/>
               </lightRig>
             </scene3d>
-            <a:sp3d>
+            <a:sp3d xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <bevelT w="63500" h="25400"/>
             </a:sp3d>
           </spPr>
@@ -3612,18 +3612,18 @@
             <dLbl>
               <idx val="8"/>
               <spPr>
-                <a:noFill/>
-                <a:ln>
+                <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:noFill/>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
                   <a:noAutofit/>
                 </a:bodyPr>
-                <a:lstStyle/>
-                <a:p>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="1100" b="0" i="0" strike="noStrike" kern="1200" baseline="0">
                       <a:solidFill>
@@ -3671,18 +3671,18 @@
               <showBubbleSize val="0"/>
             </dLbl>
             <spPr>
-              <a:noFill/>
-              <a:ln>
+              <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
             <txPr>
-              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
                 <a:spAutoFit/>
               </a:bodyPr>
-              <a:lstStyle/>
-              <a:p>
+              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr sz="1100" b="0" i="0" strike="noStrike" kern="1200" baseline="0">
                     <a:solidFill>
@@ -3815,10 +3815,10 @@
             </strRef>
           </tx>
           <spPr>
-            <a:solidFill>
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:srgbClr val="00FF00"/>
             </a:solidFill>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -3830,7 +3830,7 @@
                 <rot lat="0" lon="0" rev="1200000"/>
               </lightRig>
             </scene3d>
-            <a:sp3d>
+            <a:sp3d xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <bevelT w="63500" h="25400"/>
             </a:sp3d>
           </spPr>
@@ -3859,18 +3859,18 @@
             <dLbl>
               <idx val="3"/>
               <spPr>
-                <a:noFill/>
-                <a:ln>
+                <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:noFill/>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
                   <a:noAutofit/>
                 </a:bodyPr>
-                <a:lstStyle/>
-                <a:p>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" i="0" strike="noStrike" kern="1200" baseline="0">
                       <a:solidFill>
@@ -3920,18 +3920,18 @@
             <dLbl>
               <idx val="8"/>
               <spPr>
-                <a:noFill/>
-                <a:ln>
+                <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:noFill/>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
                   <a:noAutofit/>
                 </a:bodyPr>
-                <a:lstStyle/>
-                <a:p>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" i="0" strike="noStrike" kern="1200" baseline="0">
                       <a:solidFill>
@@ -3989,18 +3989,18 @@
               <showBubbleSize val="0"/>
             </dLbl>
             <spPr>
-              <a:noFill/>
-              <a:ln>
+              <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
             <txPr>
-              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
                 <a:spAutoFit/>
               </a:bodyPr>
-              <a:lstStyle/>
-              <a:p>
+              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr sz="1000" b="0" i="0" strike="noStrike" kern="1200" baseline="0">
                     <a:solidFill>
@@ -4133,10 +4133,10 @@
             </strRef>
           </tx>
           <spPr>
-            <a:solidFill>
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:srgbClr val="FF0000"/>
             </a:solidFill>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -4148,7 +4148,7 @@
                 <rot lat="0" lon="0" rev="1200000"/>
               </lightRig>
             </scene3d>
-            <a:sp3d>
+            <a:sp3d xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <bevelT w="63500" h="25400"/>
             </a:sp3d>
           </spPr>
@@ -4157,18 +4157,18 @@
             <dLbl>
               <idx val="3"/>
               <spPr>
-                <a:noFill/>
-                <a:ln>
+                <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:noFill/>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
                   <a:noAutofit/>
                 </a:bodyPr>
-                <a:lstStyle/>
-                <a:p>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="900" b="0" i="0" strike="noStrike" kern="1200" baseline="0">
                       <a:solidFill>
@@ -4206,18 +4206,18 @@
               <showBubbleSize val="0"/>
             </dLbl>
             <spPr>
-              <a:noFill/>
-              <a:ln>
+              <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
             <txPr>
-              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
                 <a:spAutoFit/>
               </a:bodyPr>
-              <a:lstStyle/>
-              <a:p>
+              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr sz="900" b="0" i="0" strike="noStrike" kern="1200" baseline="0">
                     <a:solidFill>
@@ -4361,8 +4361,8 @@
         <minorTickMark val="none"/>
         <tickLblPos val="nextTo"/>
         <spPr>
-          <a:noFill/>
-          <a:ln w="12700" cap="flat" cmpd="sng" algn="ctr">
+          <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12700" cap="flat" cmpd="sng" algn="ctr">
             <a:solidFill>
               <a:schemeClr val="lt1">
                 <a:alpha val="54000"/>
@@ -4374,9 +4374,9 @@
           </a:ln>
         </spPr>
         <txPr>
-          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-          <a:lstStyle/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr sz="900" b="0" i="0" strike="noStrike" kern="1200" baseline="0">
                 <a:solidFill>
@@ -4422,16 +4422,16 @@
       <legendPos val="b"/>
       <overlay val="0"/>
       <spPr>
-        <a:noFill/>
-        <a:ln>
+        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
       </spPr>
       <txPr>
-        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-        <a:lstStyle/>
-        <a:p>
+        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:pPr>
             <a:defRPr sz="900" b="0" i="0" strike="noStrike" kern="1200" baseline="0">
               <a:solidFill>
@@ -4455,7 +4455,7 @@
     <dispBlanksAs val="gap"/>
   </chart>
   <spPr>
-    <a:gradFill rotWithShape="1">
+    <a:gradFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rotWithShape="1">
       <a:gsLst>
         <a:gs pos="0">
           <a:schemeClr val="dk1">
@@ -4475,7 +4475,7 @@
       </a:path>
       <a:tileRect/>
     </a:gradFill>
-    <a:ln>
+    <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
       <a:noFill/>
       <a:prstDash val="solid"/>
     </a:ln>
@@ -4484,13 +4484,13 @@
 </file>
 
 <file path=xl/charts/chart13.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:r>
               <a:t>None</a:t>
             </a:r>
@@ -4520,7 +4520,7 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
@@ -4661,7 +4661,7 @@
 </file>
 
 <file path=xl/charts/chart14.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <plotArea>
       <layout>
@@ -4696,7 +4696,7 @@
             </strRef>
           </tx>
           <spPr>
-            <a:gradFill rotWithShape="1">
+            <a:gradFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rotWithShape="1">
               <a:gsLst>
                 <a:gs pos="0">
                   <a:schemeClr val="accent1">
@@ -4719,7 +4719,7 @@
               </a:gsLst>
               <a:lin ang="16200000" scaled="0"/>
             </a:gradFill>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -4731,7 +4731,7 @@
                 <rot lat="0" lon="0" rev="1200000"/>
               </lightRig>
             </scene3d>
-            <a:sp3d>
+            <a:sp3d xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <bevelT w="63500" h="25400"/>
             </a:sp3d>
           </spPr>
@@ -4790,18 +4790,18 @@
             <dLbl>
               <idx val="8"/>
               <spPr>
-                <a:noFill/>
-                <a:ln>
+                <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:noFill/>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
                   <a:noAutofit/>
                 </a:bodyPr>
-                <a:lstStyle/>
-                <a:p>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="1300" b="0" i="0" strike="noStrike" kern="1200" baseline="0">
                       <a:solidFill>
@@ -4849,18 +4849,18 @@
               <showBubbleSize val="0"/>
             </dLbl>
             <spPr>
-              <a:noFill/>
-              <a:ln>
+              <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
             <txPr>
-              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
                 <a:spAutoFit/>
               </a:bodyPr>
-              <a:lstStyle/>
-              <a:p>
+              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr sz="1300" b="0" i="0" strike="noStrike" kern="1200" baseline="0">
                     <a:solidFill>
@@ -4993,10 +4993,10 @@
             </strRef>
           </tx>
           <spPr>
-            <a:solidFill>
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:srgbClr val="00FF00"/>
             </a:solidFill>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -5008,7 +5008,7 @@
                 <rot lat="0" lon="0" rev="1200000"/>
               </lightRig>
             </scene3d>
-            <a:sp3d>
+            <a:sp3d xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <bevelT w="63500" h="25400"/>
             </a:sp3d>
           </spPr>
@@ -5037,18 +5037,18 @@
             <dLbl>
               <idx val="3"/>
               <spPr>
-                <a:noFill/>
-                <a:ln>
+                <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:noFill/>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
                   <a:noAutofit/>
                 </a:bodyPr>
-                <a:lstStyle/>
-                <a:p>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="1300" b="0" i="0" strike="noStrike" kern="1200" baseline="0">
                       <a:solidFill>
@@ -5098,18 +5098,18 @@
             <dLbl>
               <idx val="8"/>
               <spPr>
-                <a:noFill/>
-                <a:ln>
+                <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:noFill/>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
                   <a:noAutofit/>
                 </a:bodyPr>
-                <a:lstStyle/>
-                <a:p>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="1300" b="0" i="0" strike="noStrike" kern="1200" baseline="0">
                       <a:solidFill>
@@ -5177,18 +5177,18 @@
               <showBubbleSize val="0"/>
             </dLbl>
             <spPr>
-              <a:noFill/>
-              <a:ln>
+              <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
             <txPr>
-              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
                 <a:spAutoFit/>
               </a:bodyPr>
-              <a:lstStyle/>
-              <a:p>
+              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr sz="1300" b="0" i="0" strike="noStrike" kern="1200" baseline="0">
                     <a:solidFill>
@@ -5321,10 +5321,10 @@
             </strRef>
           </tx>
           <spPr>
-            <a:solidFill>
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:srgbClr val="FF0000"/>
             </a:solidFill>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -5336,7 +5336,7 @@
                 <rot lat="0" lon="0" rev="1200000"/>
               </lightRig>
             </scene3d>
-            <a:sp3d>
+            <a:sp3d xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <bevelT w="63500" h="25400"/>
             </a:sp3d>
           </spPr>
@@ -5345,18 +5345,18 @@
             <dLbl>
               <idx val="3"/>
               <spPr>
-                <a:noFill/>
-                <a:ln>
+                <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:noFill/>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
                   <a:noAutofit/>
                 </a:bodyPr>
-                <a:lstStyle/>
-                <a:p>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="900" b="0" i="0" strike="noStrike" kern="1200" baseline="0">
                       <a:solidFill>
@@ -5394,18 +5394,18 @@
               <showBubbleSize val="0"/>
             </dLbl>
             <spPr>
-              <a:noFill/>
-              <a:ln>
+              <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
             <txPr>
-              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
                 <a:spAutoFit/>
               </a:bodyPr>
-              <a:lstStyle/>
-              <a:p>
+              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr sz="900" b="0" i="0" strike="noStrike" kern="1200" baseline="0">
                     <a:solidFill>
@@ -5549,8 +5549,8 @@
         <minorTickMark val="none"/>
         <tickLblPos val="nextTo"/>
         <spPr>
-          <a:noFill/>
-          <a:ln w="12700" cap="flat" cmpd="sng" algn="ctr">
+          <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12700" cap="flat" cmpd="sng" algn="ctr">
             <a:solidFill>
               <a:schemeClr val="lt1">
                 <a:alpha val="54000"/>
@@ -5562,9 +5562,9 @@
           </a:ln>
         </spPr>
         <txPr>
-          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-          <a:lstStyle/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr sz="900" b="0" i="0" strike="noStrike" kern="1200" baseline="0">
                 <a:solidFill>
@@ -5610,16 +5610,16 @@
       <legendPos val="b"/>
       <overlay val="0"/>
       <spPr>
-        <a:noFill/>
-        <a:ln>
+        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
       </spPr>
       <txPr>
-        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-        <a:lstStyle/>
-        <a:p>
+        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:pPr>
             <a:defRPr sz="1200" b="0" i="0" strike="noStrike" kern="1200" baseline="0">
               <a:solidFill>
@@ -5643,7 +5643,7 @@
     <dispBlanksAs val="gap"/>
   </chart>
   <spPr>
-    <a:gradFill rotWithShape="1">
+    <a:gradFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rotWithShape="1">
       <a:gsLst>
         <a:gs pos="0">
           <a:schemeClr val="dk1">
@@ -5663,7 +5663,7 @@
       </a:path>
       <a:tileRect/>
     </a:gradFill>
-    <a:ln>
+    <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
       <a:noFill/>
       <a:prstDash val="solid"/>
     </a:ln>
@@ -5672,14 +5672,14 @@
 </file>
 
 <file path=xl/charts/chart15.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-          <a:lstStyle/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr sz="1600" b="1" i="0" strike="noStrike" kern="1200" spc="100" baseline="0">
                 <a:solidFill>
@@ -5710,16 +5710,16 @@
       </tx>
       <overlay val="0"/>
       <spPr>
-        <a:noFill/>
-        <a:ln>
+        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
       </spPr>
       <txPr>
-        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-        <a:lstStyle/>
-        <a:p>
+        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:pPr>
             <a:defRPr sz="1600" b="1" i="0" strike="noStrike" kern="1200" spc="100" baseline="0">
               <a:solidFill>
@@ -5766,7 +5766,7 @@
           <idx val="0"/>
           <order val="0"/>
           <spPr>
-            <a:gradFill rotWithShape="1">
+            <a:gradFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rotWithShape="1">
               <a:gsLst>
                 <a:gs pos="0">
                   <a:schemeClr val="accent1">
@@ -5792,7 +5792,7 @@
               </a:gsLst>
               <a:lin ang="16200000" scaled="0"/>
             </a:gradFill>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -5804,25 +5804,25 @@
                 <rot lat="0" lon="0" rev="1200000"/>
               </lightRig>
             </scene3d>
-            <a:sp3d>
+            <a:sp3d xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <bevelT w="63500" h="25400"/>
             </a:sp3d>
           </spPr>
           <invertIfNegative val="0"/>
           <dLbls>
             <spPr>
-              <a:noFill/>
-              <a:ln>
+              <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
             <txPr>
-              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
                 <a:spAutoFit/>
               </a:bodyPr>
-              <a:lstStyle/>
-              <a:p>
+              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr sz="1300" b="0" i="0" strike="noStrike" kern="1200" baseline="0">
                     <a:solidFill>
@@ -5894,7 +5894,7 @@
           <idx val="1"/>
           <order val="1"/>
           <spPr>
-            <a:gradFill rotWithShape="1">
+            <a:gradFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rotWithShape="1">
               <a:gsLst>
                 <a:gs pos="0">
                   <a:schemeClr val="accent1">
@@ -5920,7 +5920,7 @@
               </a:gsLst>
               <a:lin ang="16200000" scaled="0"/>
             </a:gradFill>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -5932,25 +5932,25 @@
                 <rot lat="0" lon="0" rev="1200000"/>
               </lightRig>
             </scene3d>
-            <a:sp3d>
+            <a:sp3d xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <bevelT w="63500" h="25400"/>
             </a:sp3d>
           </spPr>
           <invertIfNegative val="0"/>
           <dLbls>
             <spPr>
-              <a:noFill/>
-              <a:ln>
+              <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
             <txPr>
-              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
                 <a:spAutoFit/>
               </a:bodyPr>
-              <a:lstStyle/>
-              <a:p>
+              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr sz="900" b="0" i="0" strike="noStrike" kern="1200" baseline="0">
                     <a:solidFill>
@@ -6019,7 +6019,7 @@
           <idx val="2"/>
           <order val="2"/>
           <spPr>
-            <a:gradFill rotWithShape="1">
+            <a:gradFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rotWithShape="1">
               <a:gsLst>
                 <a:gs pos="0">
                   <a:schemeClr val="accent1">
@@ -6045,7 +6045,7 @@
               </a:gsLst>
               <a:lin ang="16200000" scaled="0"/>
             </a:gradFill>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -6057,25 +6057,25 @@
                 <rot lat="0" lon="0" rev="1200000"/>
               </lightRig>
             </scene3d>
-            <a:sp3d>
+            <a:sp3d xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <bevelT w="63500" h="25400"/>
             </a:sp3d>
           </spPr>
           <invertIfNegative val="0"/>
           <dLbls>
             <spPr>
-              <a:noFill/>
-              <a:ln>
+              <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
             <txPr>
-              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
                 <a:spAutoFit/>
               </a:bodyPr>
-              <a:lstStyle/>
-              <a:p>
+              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr sz="1300" b="0" i="0" strike="noStrike" kern="1200" baseline="0">
                     <a:solidFill>
@@ -6147,7 +6147,7 @@
           <idx val="3"/>
           <order val="3"/>
           <spPr>
-            <a:gradFill rotWithShape="1">
+            <a:gradFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rotWithShape="1">
               <a:gsLst>
                 <a:gs pos="0">
                   <a:schemeClr val="accent1">
@@ -6173,7 +6173,7 @@
               </a:gsLst>
               <a:lin ang="16200000" scaled="0"/>
             </a:gradFill>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -6185,25 +6185,25 @@
                 <rot lat="0" lon="0" rev="1200000"/>
               </lightRig>
             </scene3d>
-            <a:sp3d>
+            <a:sp3d xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <bevelT w="63500" h="25400"/>
             </a:sp3d>
           </spPr>
           <invertIfNegative val="0"/>
           <dLbls>
             <spPr>
-              <a:noFill/>
-              <a:ln>
+              <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
             <txPr>
-              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
                 <a:spAutoFit/>
               </a:bodyPr>
-              <a:lstStyle/>
-              <a:p>
+              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr sz="900" b="0" i="0" strike="noStrike" kern="1200" baseline="0">
                     <a:solidFill>
@@ -6272,7 +6272,7 @@
           <idx val="4"/>
           <order val="4"/>
           <spPr>
-            <a:gradFill rotWithShape="1">
+            <a:gradFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rotWithShape="1">
               <a:gsLst>
                 <a:gs pos="0">
                   <a:schemeClr val="accent1">
@@ -6298,7 +6298,7 @@
               </a:gsLst>
               <a:lin ang="16200000" scaled="0"/>
             </a:gradFill>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -6310,25 +6310,25 @@
                 <rot lat="0" lon="0" rev="1200000"/>
               </lightRig>
             </scene3d>
-            <a:sp3d>
+            <a:sp3d xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <bevelT w="63500" h="25400"/>
             </a:sp3d>
           </spPr>
           <invertIfNegative val="0"/>
           <dLbls>
             <spPr>
-              <a:noFill/>
-              <a:ln>
+              <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
             <txPr>
-              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
                 <a:spAutoFit/>
               </a:bodyPr>
-              <a:lstStyle/>
-              <a:p>
+              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr sz="1300" b="0" i="0" strike="noStrike" kern="1200" baseline="0">
                     <a:solidFill>
@@ -6400,7 +6400,7 @@
           <idx val="5"/>
           <order val="5"/>
           <spPr>
-            <a:gradFill rotWithShape="1">
+            <a:gradFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rotWithShape="1">
               <a:gsLst>
                 <a:gs pos="0">
                   <a:schemeClr val="accent1">
@@ -6423,7 +6423,7 @@
               </a:gsLst>
               <a:lin ang="16200000" scaled="0"/>
             </a:gradFill>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -6435,25 +6435,25 @@
                 <rot lat="0" lon="0" rev="1200000"/>
               </lightRig>
             </scene3d>
-            <a:sp3d>
+            <a:sp3d xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <bevelT w="63500" h="25400"/>
             </a:sp3d>
           </spPr>
           <invertIfNegative val="0"/>
           <dLbls>
             <spPr>
-              <a:noFill/>
-              <a:ln>
+              <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
             <txPr>
-              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
                 <a:spAutoFit/>
               </a:bodyPr>
-              <a:lstStyle/>
-              <a:p>
+              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr sz="900" b="0" i="0" strike="noStrike" kern="1200" baseline="0">
                     <a:solidFill>
@@ -6522,7 +6522,7 @@
           <idx val="6"/>
           <order val="6"/>
           <spPr>
-            <a:gradFill rotWithShape="1">
+            <a:gradFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rotWithShape="1">
               <a:gsLst>
                 <a:gs pos="0">
                   <a:schemeClr val="accent1">
@@ -6545,7 +6545,7 @@
               </a:gsLst>
               <a:lin ang="16200000" scaled="0"/>
             </a:gradFill>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -6557,25 +6557,25 @@
                 <rot lat="0" lon="0" rev="1200000"/>
               </lightRig>
             </scene3d>
-            <a:sp3d>
+            <a:sp3d xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <bevelT w="63500" h="25400"/>
             </a:sp3d>
           </spPr>
           <invertIfNegative val="0"/>
           <dLbls>
             <spPr>
-              <a:noFill/>
-              <a:ln>
+              <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
             <txPr>
-              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
                 <a:spAutoFit/>
               </a:bodyPr>
-              <a:lstStyle/>
-              <a:p>
+              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr sz="1300" b="0" i="0" strike="noStrike" kern="1200" baseline="0">
                     <a:solidFill>
@@ -6647,7 +6647,7 @@
           <idx val="7"/>
           <order val="7"/>
           <spPr>
-            <a:gradFill rotWithShape="1">
+            <a:gradFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rotWithShape="1">
               <a:gsLst>
                 <a:gs pos="0">
                   <a:schemeClr val="accent1">
@@ -6670,7 +6670,7 @@
               </a:gsLst>
               <a:lin ang="16200000" scaled="0"/>
             </a:gradFill>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -6682,25 +6682,25 @@
                 <rot lat="0" lon="0" rev="1200000"/>
               </lightRig>
             </scene3d>
-            <a:sp3d>
+            <a:sp3d xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <bevelT w="63500" h="25400"/>
             </a:sp3d>
           </spPr>
           <invertIfNegative val="0"/>
           <dLbls>
             <spPr>
-              <a:noFill/>
-              <a:ln>
+              <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
             <txPr>
-              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
                 <a:spAutoFit/>
               </a:bodyPr>
-              <a:lstStyle/>
-              <a:p>
+              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr sz="900" b="0" i="0" strike="noStrike" kern="1200" baseline="0">
                     <a:solidFill>
@@ -6769,7 +6769,7 @@
           <idx val="8"/>
           <order val="8"/>
           <spPr>
-            <a:gradFill rotWithShape="1">
+            <a:gradFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rotWithShape="1">
               <a:gsLst>
                 <a:gs pos="0">
                   <a:schemeClr val="accent1">
@@ -6792,7 +6792,7 @@
               </a:gsLst>
               <a:lin ang="16200000" scaled="0"/>
             </a:gradFill>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -6804,25 +6804,25 @@
                 <rot lat="0" lon="0" rev="1200000"/>
               </lightRig>
             </scene3d>
-            <a:sp3d>
+            <a:sp3d xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <bevelT w="63500" h="25400"/>
             </a:sp3d>
           </spPr>
           <invertIfNegative val="0"/>
           <dLbls>
             <spPr>
-              <a:noFill/>
-              <a:ln>
+              <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
             <txPr>
-              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
                 <a:spAutoFit/>
               </a:bodyPr>
-              <a:lstStyle/>
-              <a:p>
+              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr sz="1300" b="0" i="0" strike="noStrike" kern="1200" baseline="0">
                     <a:solidFill>
@@ -6894,7 +6894,7 @@
           <idx val="9"/>
           <order val="9"/>
           <spPr>
-            <a:gradFill rotWithShape="1">
+            <a:gradFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rotWithShape="1">
               <a:gsLst>
                 <a:gs pos="0">
                   <a:schemeClr val="accent1">
@@ -6917,7 +6917,7 @@
               </a:gsLst>
               <a:lin ang="16200000" scaled="0"/>
             </a:gradFill>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -6929,25 +6929,25 @@
                 <rot lat="0" lon="0" rev="1200000"/>
               </lightRig>
             </scene3d>
-            <a:sp3d>
+            <a:sp3d xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <bevelT w="63500" h="25400"/>
             </a:sp3d>
           </spPr>
           <invertIfNegative val="0"/>
           <dLbls>
             <spPr>
-              <a:noFill/>
-              <a:ln>
+              <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
             <txPr>
-              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
                 <a:spAutoFit/>
               </a:bodyPr>
-              <a:lstStyle/>
-              <a:p>
+              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr sz="900" b="0" i="0" strike="noStrike" kern="1200" baseline="0">
                     <a:solidFill>
@@ -7016,7 +7016,7 @@
           <idx val="10"/>
           <order val="10"/>
           <spPr>
-            <a:gradFill rotWithShape="1">
+            <a:gradFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rotWithShape="1">
               <a:gsLst>
                 <a:gs pos="0">
                   <a:schemeClr val="accent1">
@@ -7039,7 +7039,7 @@
               </a:gsLst>
               <a:lin ang="16200000" scaled="0"/>
             </a:gradFill>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -7051,25 +7051,25 @@
                 <rot lat="0" lon="0" rev="1200000"/>
               </lightRig>
             </scene3d>
-            <a:sp3d>
+            <a:sp3d xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <bevelT w="63500" h="25400"/>
             </a:sp3d>
           </spPr>
           <invertIfNegative val="0"/>
           <dLbls>
             <spPr>
-              <a:noFill/>
-              <a:ln>
+              <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
             <txPr>
-              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
                 <a:spAutoFit/>
               </a:bodyPr>
-              <a:lstStyle/>
-              <a:p>
+              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr sz="1300" b="0" i="0" strike="noStrike" kern="1200" baseline="0">
                     <a:solidFill>
@@ -7178,7 +7178,7 @@
         <axPos val="l"/>
         <majorGridlines>
           <spPr>
-            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9525" cap="flat" cmpd="sng" algn="ctr">
               <a:solidFill>
                 <a:schemeClr val="lt1">
                   <a:alpha val="10000"/>
@@ -7203,7 +7203,7 @@
     <dispBlanksAs val="gap"/>
   </chart>
   <spPr>
-    <a:gradFill rotWithShape="1">
+    <a:gradFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rotWithShape="1">
       <a:gsLst>
         <a:gs pos="0">
           <a:schemeClr val="dk1">
@@ -7223,7 +7223,7 @@
       </a:path>
       <a:tileRect/>
     </a:gradFill>
-    <a:ln>
+    <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
       <a:noFill/>
       <a:prstDash val="solid"/>
     </a:ln>
@@ -7232,14 +7232,14 @@
 </file>
 
 <file path=xl/charts/chart16.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-          <a:lstStyle/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr sz="1800" b="1" i="0" strike="noStrike" kern="1200" baseline="0">
                 <a:solidFill>
@@ -7263,16 +7263,16 @@
       </tx>
       <overlay val="0"/>
       <spPr>
-        <a:noFill/>
-        <a:ln>
+        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
       </spPr>
       <txPr>
-        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-        <a:lstStyle/>
-        <a:p>
+        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:pPr>
             <a:defRPr sz="1800" b="1" i="0" strike="noStrike" kern="1200" baseline="0">
               <a:solidFill>
@@ -7323,10 +7323,10 @@
             </strRef>
           </tx>
           <spPr>
-            <a:solidFill>
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:srgbClr val="00FF00"/>
             </a:solidFill>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -7338,7 +7338,7 @@
                 <rot lat="0" lon="0" rev="1200000"/>
               </lightRig>
             </scene3d>
-            <a:sp3d>
+            <a:sp3d xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <bevelT w="63500" h="25400"/>
             </a:sp3d>
           </spPr>
@@ -7397,18 +7397,18 @@
             <dLbl>
               <idx val="8"/>
               <spPr>
-                <a:noFill/>
-                <a:ln>
+                <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:noFill/>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
                   <a:noAutofit/>
                 </a:bodyPr>
-                <a:lstStyle/>
-                <a:p>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="1450" b="0" i="0" strike="noStrike" kern="1200" baseline="0">
                       <a:solidFill>
@@ -7456,18 +7456,18 @@
               <showBubbleSize val="0"/>
             </dLbl>
             <spPr>
-              <a:noFill/>
-              <a:ln>
+              <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
             <txPr>
-              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
                 <a:spAutoFit/>
               </a:bodyPr>
-              <a:lstStyle/>
-              <a:p>
+              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr sz="1450" b="0" i="0" strike="noStrike" kern="1200" baseline="0">
                     <a:solidFill>
@@ -7571,10 +7571,10 @@
             </strRef>
           </tx>
           <spPr>
-            <a:solidFill>
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:srgbClr val="FF0000"/>
             </a:solidFill>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -7642,18 +7642,18 @@
               <showBubbleSize val="0"/>
             </dLbl>
             <spPr>
-              <a:noFill/>
-              <a:ln>
+              <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
             <txPr>
-              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
                 <a:spAutoFit/>
               </a:bodyPr>
-              <a:lstStyle/>
-              <a:p>
+              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr sz="1300" b="0" i="0" strike="noStrike" kern="1200" baseline="0">
                     <a:solidFill>
@@ -7766,8 +7766,8 @@
         <minorTickMark val="none"/>
         <tickLblPos val="nextTo"/>
         <spPr>
-          <a:noFill/>
-          <a:ln w="12700" cap="flat" cmpd="sng" algn="ctr">
+          <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12700" cap="flat" cmpd="sng" algn="ctr">
             <a:solidFill>
               <a:schemeClr val="lt1">
                 <a:alpha val="54000"/>
@@ -7779,9 +7779,9 @@
           </a:ln>
         </spPr>
         <txPr>
-          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-          <a:lstStyle/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr sz="1500" b="0" i="0" strike="noStrike" kern="1200" baseline="0">
                 <a:solidFill>
@@ -7827,16 +7827,16 @@
       <legendPos val="b"/>
       <overlay val="0"/>
       <spPr>
-        <a:noFill/>
-        <a:ln>
+        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
       </spPr>
       <txPr>
-        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-        <a:lstStyle/>
-        <a:p>
+        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:pPr>
             <a:defRPr sz="900" b="0" i="0" strike="noStrike" kern="1200" baseline="0">
               <a:solidFill>
@@ -7860,7 +7860,7 @@
     <dispBlanksAs val="gap"/>
   </chart>
   <spPr>
-    <a:gradFill rotWithShape="1">
+    <a:gradFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rotWithShape="1">
       <a:gsLst>
         <a:gs pos="0">
           <a:schemeClr val="dk1">
@@ -7880,7 +7880,7 @@
       </a:path>
       <a:tileRect/>
     </a:gradFill>
-    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+    <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9525" cap="flat" cmpd="sng" algn="ctr">
       <a:noFill/>
       <a:prstDash val="solid"/>
       <a:round/>
@@ -7890,7 +7890,7 @@
 </file>
 
 <file path=xl/charts/chart17.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <plotArea>
       <layout>
@@ -7925,10 +7925,10 @@
             </strRef>
           </tx>
           <spPr>
-            <a:solidFill>
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:srgbClr val="00FF00"/>
             </a:solidFill>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -7940,7 +7940,7 @@
                 <rot lat="0" lon="0" rev="1200000"/>
               </lightRig>
             </scene3d>
-            <a:sp3d>
+            <a:sp3d xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <bevelT w="63500" h="25400"/>
             </a:sp3d>
           </spPr>
@@ -8009,18 +8009,18 @@
             <dLbl>
               <idx val="8"/>
               <spPr>
-                <a:noFill/>
-                <a:ln>
+                <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:noFill/>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
                   <a:noAutofit/>
                 </a:bodyPr>
-                <a:lstStyle/>
-                <a:p>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="1300" b="0" i="0" strike="noStrike" kern="1200" baseline="0">
                       <a:solidFill>
@@ -8068,18 +8068,18 @@
               <showBubbleSize val="0"/>
             </dLbl>
             <spPr>
-              <a:noFill/>
-              <a:ln>
+              <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
             <txPr>
-              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
                 <a:spAutoFit/>
               </a:bodyPr>
-              <a:lstStyle/>
-              <a:p>
+              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr sz="1300" b="0" i="0" strike="noStrike" kern="1200" baseline="0">
                     <a:solidFill>
@@ -8191,10 +8191,10 @@
             </strRef>
           </tx>
           <spPr>
-            <a:solidFill>
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:srgbClr val="FF0000"/>
             </a:solidFill>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -8206,7 +8206,7 @@
                 <rot lat="0" lon="0" rev="1200000"/>
               </lightRig>
             </scene3d>
-            <a:sp3d>
+            <a:sp3d xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <bevelT w="63500" h="25400"/>
             </a:sp3d>
           </spPr>
@@ -8215,18 +8215,18 @@
             <dLbl>
               <idx val="3"/>
               <spPr>
-                <a:noFill/>
-                <a:ln>
+                <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:noFill/>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
                   <a:noAutofit/>
                 </a:bodyPr>
-                <a:lstStyle/>
-                <a:p>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="1020" b="0" i="0" strike="noStrike" kern="1200" baseline="0">
                       <a:solidFill>
@@ -8264,18 +8264,18 @@
               <showBubbleSize val="0"/>
             </dLbl>
             <spPr>
-              <a:noFill/>
-              <a:ln>
+              <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
             <txPr>
-              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
                 <a:spAutoFit/>
               </a:bodyPr>
-              <a:lstStyle/>
-              <a:p>
+              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr sz="1020" b="0" i="0" strike="noStrike" kern="1200" baseline="0">
                     <a:solidFill>
@@ -8398,8 +8398,8 @@
         <minorTickMark val="none"/>
         <tickLblPos val="nextTo"/>
         <spPr>
-          <a:noFill/>
-          <a:ln w="12700" cap="flat" cmpd="sng" algn="ctr">
+          <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12700" cap="flat" cmpd="sng" algn="ctr">
             <a:solidFill>
               <a:schemeClr val="lt1">
                 <a:alpha val="54000"/>
@@ -8411,9 +8411,9 @@
           </a:ln>
         </spPr>
         <txPr>
-          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-          <a:lstStyle/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr sz="900" b="0" i="0" strike="noStrike" kern="1200" baseline="0">
                 <a:solidFill>
@@ -8459,16 +8459,16 @@
       <legendPos val="b"/>
       <overlay val="0"/>
       <spPr>
-        <a:noFill/>
-        <a:ln>
+        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
       </spPr>
       <txPr>
-        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-        <a:lstStyle/>
-        <a:p>
+        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:pPr>
             <a:defRPr sz="1200" b="0" i="0" strike="noStrike" kern="1200" baseline="0">
               <a:solidFill>
@@ -8492,7 +8492,7 @@
     <dispBlanksAs val="gap"/>
   </chart>
   <spPr>
-    <a:gradFill rotWithShape="1">
+    <a:gradFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rotWithShape="1">
       <a:gsLst>
         <a:gs pos="0">
           <a:schemeClr val="dk1">
@@ -8512,7 +8512,7 @@
       </a:path>
       <a:tileRect/>
     </a:gradFill>
-    <a:ln>
+    <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
       <a:noFill/>
       <a:prstDash val="solid"/>
     </a:ln>
@@ -8521,14 +8521,14 @@
 </file>
 
 <file path=xl/charts/chart18.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-          <a:lstStyle/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr sz="1600" b="1" i="0" strike="noStrike" kern="1200" spc="100" baseline="0">
                 <a:solidFill>
@@ -8559,16 +8559,16 @@
       </tx>
       <overlay val="0"/>
       <spPr>
-        <a:noFill/>
-        <a:ln>
+        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
       </spPr>
       <txPr>
-        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-        <a:lstStyle/>
-        <a:p>
+        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:pPr>
             <a:defRPr sz="1600" b="1" i="0" strike="noStrike" kern="1200" spc="100" baseline="0">
               <a:solidFill>
@@ -8615,7 +8615,7 @@
           <idx val="0"/>
           <order val="0"/>
           <spPr>
-            <a:gradFill rotWithShape="1">
+            <a:gradFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rotWithShape="1">
               <a:gsLst>
                 <a:gs pos="0">
                   <a:schemeClr val="accent1">
@@ -8638,7 +8638,7 @@
               </a:gsLst>
               <a:lin ang="16200000" scaled="0"/>
             </a:gradFill>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -8650,25 +8650,25 @@
                 <rot lat="0" lon="0" rev="1200000"/>
               </lightRig>
             </scene3d>
-            <a:sp3d>
+            <a:sp3d xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <bevelT w="63500" h="25400"/>
             </a:sp3d>
           </spPr>
           <invertIfNegative val="0"/>
           <dLbls>
             <spPr>
-              <a:noFill/>
-              <a:ln>
+              <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
             <txPr>
-              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
                 <a:spAutoFit/>
               </a:bodyPr>
-              <a:lstStyle/>
-              <a:p>
+              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr sz="2000" b="0" i="0" strike="noStrike" kern="1200" baseline="0">
                     <a:solidFill>
@@ -8767,7 +8767,7 @@
         <axPos val="l"/>
         <majorGridlines>
           <spPr>
-            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9525" cap="flat" cmpd="sng" algn="ctr">
               <a:solidFill>
                 <a:schemeClr val="lt1">
                   <a:alpha val="10000"/>
@@ -8792,7 +8792,7 @@
     <dispBlanksAs val="gap"/>
   </chart>
   <spPr>
-    <a:gradFill rotWithShape="1">
+    <a:gradFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rotWithShape="1">
       <a:gsLst>
         <a:gs pos="0">
           <a:schemeClr val="dk1">
@@ -8812,7 +8812,7 @@
       </a:path>
       <a:tileRect/>
     </a:gradFill>
-    <a:ln>
+    <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
       <a:noFill/>
       <a:prstDash val="solid"/>
     </a:ln>
@@ -8821,14 +8821,14 @@
 </file>
 
 <file path=xl/charts/chart19.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-          <a:lstStyle/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr sz="1800" b="1" i="0" strike="noStrike" kern="1200" baseline="0">
                 <a:solidFill>
@@ -8852,16 +8852,16 @@
       </tx>
       <overlay val="0"/>
       <spPr>
-        <a:noFill/>
-        <a:ln>
+        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
       </spPr>
       <txPr>
-        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-        <a:lstStyle/>
-        <a:p>
+        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:pPr>
             <a:defRPr sz="1800" b="1" i="0" strike="noStrike" kern="1200" baseline="0">
               <a:solidFill>
@@ -8912,10 +8912,10 @@
             </strRef>
           </tx>
           <spPr>
-            <a:solidFill>
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:srgbClr val="00FF00"/>
             </a:solidFill>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -8927,7 +8927,7 @@
                 <rot lat="0" lon="0" rev="1200000"/>
               </lightRig>
             </scene3d>
-            <a:sp3d>
+            <a:sp3d xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <bevelT w="63500" h="25400"/>
             </a:sp3d>
           </spPr>
@@ -8986,18 +8986,18 @@
             <dLbl>
               <idx val="8"/>
               <spPr>
-                <a:noFill/>
-                <a:ln>
+                <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:noFill/>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
                   <a:noAutofit/>
                 </a:bodyPr>
-                <a:lstStyle/>
-                <a:p>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="1450" b="0" i="0" strike="noStrike" kern="1200" baseline="0">
                       <a:solidFill>
@@ -9045,18 +9045,18 @@
               <showBubbleSize val="0"/>
             </dLbl>
             <spPr>
-              <a:noFill/>
-              <a:ln>
+              <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
             <txPr>
-              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
                 <a:spAutoFit/>
               </a:bodyPr>
-              <a:lstStyle/>
-              <a:p>
+              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr sz="1450" b="0" i="0" strike="noStrike" kern="1200" baseline="0">
                     <a:solidFill>
@@ -9160,10 +9160,10 @@
             </strRef>
           </tx>
           <spPr>
-            <a:solidFill>
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:srgbClr val="FF0000"/>
             </a:solidFill>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -9231,18 +9231,18 @@
               <showBubbleSize val="0"/>
             </dLbl>
             <spPr>
-              <a:noFill/>
-              <a:ln>
+              <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
             <txPr>
-              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
                 <a:spAutoFit/>
               </a:bodyPr>
-              <a:lstStyle/>
-              <a:p>
+              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr sz="1300" b="0" i="0" strike="noStrike" kern="1200" baseline="0">
                     <a:solidFill>
@@ -9355,8 +9355,8 @@
         <minorTickMark val="none"/>
         <tickLblPos val="nextTo"/>
         <spPr>
-          <a:noFill/>
-          <a:ln w="12700" cap="flat" cmpd="sng" algn="ctr">
+          <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12700" cap="flat" cmpd="sng" algn="ctr">
             <a:solidFill>
               <a:schemeClr val="lt1">
                 <a:alpha val="54000"/>
@@ -9368,9 +9368,9 @@
           </a:ln>
         </spPr>
         <txPr>
-          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-          <a:lstStyle/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr sz="1500" b="0" i="0" strike="noStrike" kern="1200" baseline="0">
                 <a:solidFill>
@@ -9416,16 +9416,16 @@
       <legendPos val="b"/>
       <overlay val="0"/>
       <spPr>
-        <a:noFill/>
-        <a:ln>
+        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
       </spPr>
       <txPr>
-        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-        <a:lstStyle/>
-        <a:p>
+        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:pPr>
             <a:defRPr sz="900" b="0" i="0" strike="noStrike" kern="1200" baseline="0">
               <a:solidFill>
@@ -9449,7 +9449,7 @@
     <dispBlanksAs val="gap"/>
   </chart>
   <spPr>
-    <a:gradFill rotWithShape="1">
+    <a:gradFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rotWithShape="1">
       <a:gsLst>
         <a:gs pos="0">
           <a:schemeClr val="dk1">
@@ -9469,7 +9469,7 @@
       </a:path>
       <a:tileRect/>
     </a:gradFill>
-    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+    <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9525" cap="flat" cmpd="sng" algn="ctr">
       <a:noFill/>
       <a:prstDash val="solid"/>
       <a:round/>
@@ -9479,14 +9479,14 @@
 </file>
 
 <file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-          <a:lstStyle/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr sz="1600" b="1" i="0" strike="noStrike" kern="1200" spc="100" baseline="0">
                 <a:solidFill>
@@ -9526,16 +9526,16 @@
       </tx>
       <overlay val="0"/>
       <spPr>
-        <a:noFill/>
-        <a:ln>
+        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
       </spPr>
       <txPr>
-        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-        <a:lstStyle/>
-        <a:p>
+        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:pPr>
             <a:defRPr sz="1600" b="1" i="0" strike="noStrike" kern="1200" spc="100" baseline="0">
               <a:solidFill>
@@ -9593,10 +9593,10 @@
             </strRef>
           </tx>
           <spPr>
-            <a:solidFill>
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:srgbClr val="00CC00"/>
             </a:solidFill>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -9608,25 +9608,25 @@
                 <rot lat="0" lon="0" rev="1200000"/>
               </lightRig>
             </scene3d>
-            <a:sp3d>
+            <a:sp3d xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <bevelT w="63500" h="25400"/>
             </a:sp3d>
           </spPr>
           <invertIfNegative val="0"/>
           <dLbls>
             <spPr>
-              <a:noFill/>
-              <a:ln>
+              <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
             <txPr>
-              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
                 <a:spAutoFit/>
               </a:bodyPr>
-              <a:lstStyle/>
-              <a:p>
+              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr sz="1200" b="0" i="0" strike="noStrike" kern="1200" baseline="0">
                     <a:solidFill>
@@ -9695,10 +9695,10 @@
             </strRef>
           </tx>
           <spPr>
-            <a:solidFill>
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:srgbClr val="32C1FA"/>
             </a:solidFill>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -9710,25 +9710,25 @@
                 <rot lat="0" lon="0" rev="1200000"/>
               </lightRig>
             </scene3d>
-            <a:sp3d>
+            <a:sp3d xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <bevelT w="63500" h="25400"/>
             </a:sp3d>
           </spPr>
           <invertIfNegative val="0"/>
           <dLbls>
             <spPr>
-              <a:noFill/>
-              <a:ln>
+              <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
             <txPr>
-              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
                 <a:spAutoFit/>
               </a:bodyPr>
-              <a:lstStyle/>
-              <a:p>
+              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr sz="1200" b="0" i="0" strike="noStrike" kern="1200" baseline="0">
                     <a:solidFill>
@@ -9797,10 +9797,10 @@
             </strRef>
           </tx>
           <spPr>
-            <a:solidFill>
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:srgbClr val="FF0000"/>
             </a:solidFill>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -9812,25 +9812,25 @@
                 <rot lat="0" lon="0" rev="1200000"/>
               </lightRig>
             </scene3d>
-            <a:sp3d>
+            <a:sp3d xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <bevelT w="63500" h="25400"/>
             </a:sp3d>
           </spPr>
           <invertIfNegative val="0"/>
           <dLbls>
             <spPr>
-              <a:noFill/>
-              <a:ln>
+              <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
             <txPr>
-              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
                 <a:spAutoFit/>
               </a:bodyPr>
-              <a:lstStyle/>
-              <a:p>
+              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr sz="1200" b="0" i="0" strike="noStrike" kern="1200" baseline="0">
                     <a:solidFill>
@@ -9926,16 +9926,16 @@
         <minorTickMark val="none"/>
         <tickLblPos val="nextTo"/>
         <spPr>
-          <a:noFill/>
-          <a:ln>
+          <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:noFill/>
             <a:prstDash val="solid"/>
           </a:ln>
         </spPr>
         <txPr>
-          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-          <a:lstStyle/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr sz="900" b="0" i="0" strike="noStrike" kern="1200" baseline="0">
                 <a:solidFill>
@@ -9963,7 +9963,7 @@
     <dispBlanksAs val="gap"/>
   </chart>
   <spPr>
-    <a:gradFill rotWithShape="1">
+    <a:gradFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rotWithShape="1">
       <a:gsLst>
         <a:gs pos="0">
           <a:schemeClr val="dk1">
@@ -9983,7 +9983,7 @@
       </a:path>
       <a:tileRect/>
     </a:gradFill>
-    <a:ln>
+    <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
       <a:noFill/>
       <a:prstDash val="solid"/>
     </a:ln>
@@ -9992,14 +9992,14 @@
 </file>
 
 <file path=xl/charts/chart20.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-          <a:lstStyle/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr sz="1600" b="1" i="0" strike="noStrike" kern="1200" spc="100" baseline="0">
                 <a:solidFill>
@@ -10030,16 +10030,16 @@
       </tx>
       <overlay val="0"/>
       <spPr>
-        <a:noFill/>
-        <a:ln>
+        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
       </spPr>
       <txPr>
-        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-        <a:lstStyle/>
-        <a:p>
+        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:pPr>
             <a:defRPr sz="1600" b="1" i="0" strike="noStrike" kern="1200" spc="100" baseline="0">
               <a:solidFill>
@@ -10086,7 +10086,7 @@
           <idx val="0"/>
           <order val="0"/>
           <spPr>
-            <a:gradFill rotWithShape="1">
+            <a:gradFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rotWithShape="1">
               <a:gsLst>
                 <a:gs pos="0">
                   <a:schemeClr val="accent1">
@@ -10109,7 +10109,7 @@
               </a:gsLst>
               <a:lin ang="16200000" scaled="0"/>
             </a:gradFill>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -10121,25 +10121,25 @@
                 <rot lat="0" lon="0" rev="1200000"/>
               </lightRig>
             </scene3d>
-            <a:sp3d>
+            <a:sp3d xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <bevelT w="63500" h="25400"/>
             </a:sp3d>
           </spPr>
           <invertIfNegative val="0"/>
           <dLbls>
             <spPr>
-              <a:noFill/>
-              <a:ln>
+              <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
             <txPr>
-              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
                 <a:spAutoFit/>
               </a:bodyPr>
-              <a:lstStyle/>
-              <a:p>
+              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr sz="1500" b="0" i="0" strike="noStrike" kern="1200" baseline="0">
                     <a:solidFill>
@@ -10431,7 +10431,7 @@
         <axPos val="l"/>
         <majorGridlines>
           <spPr>
-            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9525" cap="flat" cmpd="sng" algn="ctr">
               <a:solidFill>
                 <a:schemeClr val="lt1">
                   <a:alpha val="10000"/>
@@ -10456,7 +10456,7 @@
     <dispBlanksAs val="gap"/>
   </chart>
   <spPr>
-    <a:gradFill rotWithShape="1">
+    <a:gradFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rotWithShape="1">
       <a:gsLst>
         <a:gs pos="0">
           <a:schemeClr val="dk1">
@@ -10476,7 +10476,7 @@
       </a:path>
       <a:tileRect/>
     </a:gradFill>
-    <a:ln>
+    <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
       <a:noFill/>
       <a:prstDash val="solid"/>
     </a:ln>
@@ -10485,7 +10485,7 @@
 </file>
 
 <file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <plotArea>
       <layout>
@@ -10520,7 +10520,7 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
@@ -10618,7 +10618,7 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
@@ -10759,14 +10759,14 @@
 </file>
 
 <file path=xl/charts/chart4.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr/>
-          <a:lstStyle/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr/>
             </a:pPr>
@@ -10800,7 +10800,7 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
@@ -10921,8 +10921,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:r>
                   <a:t>None</a:t>
                 </a:r>
@@ -10951,13 +10951,13 @@
 </file>
 
 <file path=xl/charts/chart5.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:r>
               <a:t>None</a:t>
             </a:r>
@@ -10987,7 +10987,7 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
@@ -11128,7 +11128,7 @@
 </file>
 
 <file path=xl/charts/chart6.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <plotArea>
       <layout>
@@ -11163,7 +11163,7 @@
             </strRef>
           </tx>
           <spPr>
-            <a:gradFill rotWithShape="1">
+            <a:gradFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rotWithShape="1">
               <a:gsLst>
                 <a:gs pos="0">
                   <a:schemeClr val="accent1">
@@ -11186,7 +11186,7 @@
               </a:gsLst>
               <a:lin ang="16200000" scaled="0"/>
             </a:gradFill>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -11198,7 +11198,7 @@
                 <rot lat="0" lon="0" rev="1200000"/>
               </lightRig>
             </scene3d>
-            <a:sp3d>
+            <a:sp3d xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <bevelT w="63500" h="25400"/>
             </a:sp3d>
           </spPr>
@@ -11215,18 +11215,18 @@
               <showBubbleSize val="0"/>
             </dLbl>
             <spPr>
-              <a:noFill/>
-              <a:ln>
+              <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
             <txPr>
-              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
                 <a:spAutoFit/>
               </a:bodyPr>
-              <a:lstStyle/>
-              <a:p>
+              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr sz="1100" b="0" i="0" strike="noStrike" kern="1200" baseline="0">
                     <a:solidFill>
@@ -11359,10 +11359,10 @@
             </strRef>
           </tx>
           <spPr>
-            <a:solidFill>
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:srgbClr val="00FF00"/>
             </a:solidFill>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -11374,7 +11374,7 @@
                 <rot lat="0" lon="0" rev="1200000"/>
               </lightRig>
             </scene3d>
-            <a:sp3d>
+            <a:sp3d xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <bevelT w="63500" h="25400"/>
             </a:sp3d>
           </spPr>
@@ -11391,18 +11391,18 @@
               <showBubbleSize val="0"/>
             </dLbl>
             <spPr>
-              <a:noFill/>
-              <a:ln>
+              <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
             <txPr>
-              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
                 <a:spAutoFit/>
               </a:bodyPr>
-              <a:lstStyle/>
-              <a:p>
+              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr sz="1000" b="0" i="0" strike="noStrike" kern="1200" baseline="0">
                     <a:solidFill>
@@ -11535,10 +11535,10 @@
             </strRef>
           </tx>
           <spPr>
-            <a:solidFill>
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:srgbClr val="FF0000"/>
             </a:solidFill>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -11550,25 +11550,25 @@
                 <rot lat="0" lon="0" rev="1200000"/>
               </lightRig>
             </scene3d>
-            <a:sp3d>
+            <a:sp3d xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <bevelT w="63500" h="25400"/>
             </a:sp3d>
           </spPr>
           <invertIfNegative val="0"/>
           <dLbls>
             <spPr>
-              <a:noFill/>
-              <a:ln>
+              <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
             <txPr>
-              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
                 <a:spAutoFit/>
               </a:bodyPr>
-              <a:lstStyle/>
-              <a:p>
+              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr sz="900" b="0" i="0" strike="noStrike" kern="1200" baseline="0">
                     <a:solidFill>
@@ -11712,8 +11712,8 @@
         <minorTickMark val="none"/>
         <tickLblPos val="nextTo"/>
         <spPr>
-          <a:noFill/>
-          <a:ln w="12700" cap="flat" cmpd="sng" algn="ctr">
+          <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12700" cap="flat" cmpd="sng" algn="ctr">
             <a:solidFill>
               <a:schemeClr val="lt1">
                 <a:alpha val="54000"/>
@@ -11725,9 +11725,9 @@
           </a:ln>
         </spPr>
         <txPr>
-          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-          <a:lstStyle/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr sz="900" b="0" i="0" strike="noStrike" kern="1200" baseline="0">
                 <a:solidFill>
@@ -11773,16 +11773,16 @@
       <legendPos val="b"/>
       <overlay val="0"/>
       <spPr>
-        <a:noFill/>
-        <a:ln>
+        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
       </spPr>
       <txPr>
-        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-        <a:lstStyle/>
-        <a:p>
+        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:pPr>
             <a:defRPr sz="900" b="0" i="0" strike="noStrike" kern="1200" baseline="0">
               <a:solidFill>
@@ -11806,7 +11806,7 @@
     <dispBlanksAs val="gap"/>
   </chart>
   <spPr>
-    <a:gradFill rotWithShape="1">
+    <a:gradFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rotWithShape="1">
       <a:gsLst>
         <a:gs pos="0">
           <a:schemeClr val="dk1">
@@ -11826,7 +11826,7 @@
       </a:path>
       <a:tileRect/>
     </a:gradFill>
-    <a:ln>
+    <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
       <a:noFill/>
       <a:prstDash val="solid"/>
     </a:ln>
@@ -11835,13 +11835,13 @@
 </file>
 
 <file path=xl/charts/chart7.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:r>
               <a:t>None</a:t>
             </a:r>
@@ -11871,7 +11871,7 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
@@ -12006,7 +12006,7 @@
 </file>
 
 <file path=xl/charts/chart8.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <plotArea>
       <layout>
@@ -12041,7 +12041,7 @@
             </strRef>
           </tx>
           <spPr>
-            <a:gradFill rotWithShape="1">
+            <a:gradFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rotWithShape="1">
               <a:gsLst>
                 <a:gs pos="0">
                   <a:schemeClr val="accent1">
@@ -12064,7 +12064,7 @@
               </a:gsLst>
               <a:lin ang="16200000" scaled="0"/>
             </a:gradFill>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -12076,7 +12076,7 @@
                 <rot lat="0" lon="0" rev="1200000"/>
               </lightRig>
             </scene3d>
-            <a:sp3d>
+            <a:sp3d xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <bevelT w="63500" h="25400"/>
             </a:sp3d>
           </spPr>
@@ -12143,18 +12143,18 @@
               <showBubbleSize val="0"/>
             </dLbl>
             <spPr>
-              <a:noFill/>
-              <a:ln>
+              <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
             <txPr>
-              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
                 <a:spAutoFit/>
               </a:bodyPr>
-              <a:lstStyle/>
-              <a:p>
+              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr sz="1100" b="0" i="0" strike="noStrike" kern="1200" baseline="0">
                     <a:solidFill>
@@ -12287,10 +12287,10 @@
             </strRef>
           </tx>
           <spPr>
-            <a:solidFill>
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:srgbClr val="00FF00"/>
             </a:solidFill>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -12302,7 +12302,7 @@
                 <rot lat="0" lon="0" rev="1200000"/>
               </lightRig>
             </scene3d>
-            <a:sp3d>
+            <a:sp3d xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <bevelT w="63500" h="25400"/>
             </a:sp3d>
           </spPr>
@@ -12349,18 +12349,18 @@
               <showBubbleSize val="0"/>
             </dLbl>
             <spPr>
-              <a:noFill/>
-              <a:ln>
+              <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
             <txPr>
-              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
                 <a:spAutoFit/>
               </a:bodyPr>
-              <a:lstStyle/>
-              <a:p>
+              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr sz="1000" b="0" i="0" strike="noStrike" kern="1200" baseline="0">
                     <a:solidFill>
@@ -12493,10 +12493,10 @@
             </strRef>
           </tx>
           <spPr>
-            <a:solidFill>
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:srgbClr val="FF0000"/>
             </a:solidFill>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -12508,7 +12508,7 @@
                 <rot lat="0" lon="0" rev="1200000"/>
               </lightRig>
             </scene3d>
-            <a:sp3d>
+            <a:sp3d xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <bevelT w="63500" h="25400"/>
             </a:sp3d>
           </spPr>
@@ -12525,18 +12525,18 @@
               <showBubbleSize val="0"/>
             </dLbl>
             <spPr>
-              <a:noFill/>
-              <a:ln>
+              <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
             <txPr>
-              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
                 <a:spAutoFit/>
               </a:bodyPr>
-              <a:lstStyle/>
-              <a:p>
+              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr sz="900" b="0" i="0" strike="noStrike" kern="1200" baseline="0">
                     <a:solidFill>
@@ -12671,8 +12671,8 @@
         <minorTickMark val="none"/>
         <tickLblPos val="nextTo"/>
         <spPr>
-          <a:noFill/>
-          <a:ln w="12700" cap="flat" cmpd="sng" algn="ctr">
+          <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12700" cap="flat" cmpd="sng" algn="ctr">
             <a:solidFill>
               <a:schemeClr val="lt1">
                 <a:alpha val="54000"/>
@@ -12684,9 +12684,9 @@
           </a:ln>
         </spPr>
         <txPr>
-          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-          <a:lstStyle/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr sz="900" b="0" i="0" strike="noStrike" kern="1200" baseline="0">
                 <a:solidFill>
@@ -12732,16 +12732,16 @@
       <legendPos val="b"/>
       <overlay val="0"/>
       <spPr>
-        <a:noFill/>
-        <a:ln>
+        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
       </spPr>
       <txPr>
-        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-        <a:lstStyle/>
-        <a:p>
+        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:pPr>
             <a:defRPr sz="900" b="0" i="0" strike="noStrike" kern="1200" baseline="0">
               <a:solidFill>
@@ -12765,7 +12765,7 @@
     <dispBlanksAs val="gap"/>
   </chart>
   <spPr>
-    <a:gradFill rotWithShape="1">
+    <a:gradFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rotWithShape="1">
       <a:gsLst>
         <a:gs pos="0">
           <a:schemeClr val="dk1">
@@ -12785,7 +12785,7 @@
       </a:path>
       <a:tileRect/>
     </a:gradFill>
-    <a:ln>
+    <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
       <a:noFill/>
       <a:prstDash val="solid"/>
     </a:ln>
@@ -12794,13 +12794,13 @@
 </file>
 
 <file path=xl/charts/chart9.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:r>
               <a:t>None</a:t>
             </a:r>
@@ -12830,7 +12830,7 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
@@ -13013,7 +13013,7 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <twoCellAnchor>
     <from>
       <col>5</col>
@@ -13033,9 +13033,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId1"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -13060,9 +13060,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId2"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -13072,7 +13072,7 @@
 </file>
 
 <file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <twoCellAnchor>
     <from>
       <col>5</col>
@@ -13092,9 +13092,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId1"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -13119,9 +13119,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId2"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -13146,9 +13146,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId3"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId3"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -13171,24 +13171,24 @@
       <nvPicPr>
         <cNvPr id="2" name="Imagem 1" descr="logo_red.png"/>
         <cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
+          <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
         </cNvPicPr>
       </nvPicPr>
       <blipFill>
-        <a:blip r:embed="rId4"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId4"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:xfrm>
+        <a:xfrm xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:off x="702945" y="238124"/>
           <a:ext cx="4133970" cy="771525"/>
         </a:xfrm>
-        <a:prstGeom prst="rect">
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect">
           <avLst/>
         </a:prstGeom>
-        <a:ln>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:prstDash val="solid"/>
         </a:ln>
       </spPr>
@@ -13199,7 +13199,7 @@
 </file>
 
 <file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <twoCellAnchor>
     <from>
       <col>6</col>
@@ -13219,9 +13219,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId1"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -13246,9 +13246,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId2"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -13271,24 +13271,24 @@
       <nvPicPr>
         <cNvPr id="2" name="Imagem 1" descr="logo_red.png"/>
         <cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
+          <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
         </cNvPicPr>
       </nvPicPr>
       <blipFill>
-        <a:blip r:embed="rId3"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId3"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:xfrm>
+        <a:xfrm xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:off x="331468" y="207166"/>
           <a:ext cx="6154538" cy="1138239"/>
         </a:xfrm>
-        <a:prstGeom prst="rect">
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect">
           <avLst/>
         </a:prstGeom>
-        <a:ln>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:prstDash val="solid"/>
         </a:ln>
       </spPr>
@@ -13299,7 +13299,7 @@
 </file>
 
 <file path=xl/drawings/drawing4.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <twoCellAnchor>
     <from>
       <col>6</col>
@@ -13319,9 +13319,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId1"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -13346,9 +13346,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId2"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -13371,24 +13371,24 @@
       <nvPicPr>
         <cNvPr id="2" name="Imagem 1" descr="logo_red.png"/>
         <cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
+          <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
         </cNvPicPr>
       </nvPicPr>
       <blipFill>
-        <a:blip r:embed="rId3"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId3"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:xfrm>
+        <a:xfrm xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:off x="331468" y="390524"/>
           <a:ext cx="3735707" cy="741509"/>
         </a:xfrm>
-        <a:prstGeom prst="rect">
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect">
           <avLst/>
         </a:prstGeom>
-        <a:ln>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:prstDash val="solid"/>
         </a:ln>
       </spPr>
@@ -13399,7 +13399,7 @@
 </file>
 
 <file path=xl/drawings/drawing5.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <twoCellAnchor>
     <from>
       <col>6</col>
@@ -13419,9 +13419,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId1"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -13446,9 +13446,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId2"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -13471,24 +13471,24 @@
       <nvPicPr>
         <cNvPr id="2" name="Imagem 1" descr="logo_red.png"/>
         <cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
+          <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
         </cNvPicPr>
       </nvPicPr>
       <blipFill>
-        <a:blip r:embed="rId3"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId3"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:xfrm>
+        <a:xfrm xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:off x="560068" y="380999"/>
           <a:ext cx="3157563" cy="676276"/>
         </a:xfrm>
-        <a:prstGeom prst="rect">
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect">
           <avLst/>
         </a:prstGeom>
-        <a:ln>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:prstDash val="solid"/>
         </a:ln>
       </spPr>
@@ -13499,7 +13499,7 @@
 </file>
 
 <file path=xl/drawings/drawing6.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <twoCellAnchor>
     <from>
       <col>5</col>
@@ -13519,9 +13519,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId1"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -13546,9 +13546,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId2"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -13571,24 +13571,24 @@
       <nvPicPr>
         <cNvPr id="2" name="Imagem 1" descr="logo_red.png"/>
         <cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
+          <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
         </cNvPicPr>
       </nvPicPr>
       <blipFill>
-        <a:blip r:embed="rId3"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId3"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:xfrm>
+        <a:xfrm xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:off x="3072286" y="280987"/>
           <a:ext cx="4238151" cy="754857"/>
         </a:xfrm>
-        <a:prstGeom prst="rect">
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect">
           <avLst/>
         </a:prstGeom>
-        <a:ln>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:prstDash val="solid"/>
         </a:ln>
       </spPr>
@@ -13599,7 +13599,7 @@
 </file>
 
 <file path=xl/drawings/drawing7.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <twoCellAnchor>
     <from>
       <col>5</col>
@@ -13619,9 +13619,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId1"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -13646,9 +13646,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId2"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -13673,9 +13673,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId3"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId3"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -13698,24 +13698,24 @@
       <nvPicPr>
         <cNvPr id="2" name="Imagem 1" descr="logo_red.png"/>
         <cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
+          <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
         </cNvPicPr>
       </nvPicPr>
       <blipFill>
-        <a:blip r:embed="rId4"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId4"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:xfrm>
+        <a:xfrm xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:off x="3127531" y="285273"/>
           <a:ext cx="4356261" cy="744380"/>
         </a:xfrm>
-        <a:prstGeom prst="rect">
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect">
           <avLst/>
         </a:prstGeom>
-        <a:ln>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:prstDash val="solid"/>
         </a:ln>
       </spPr>
@@ -13726,7 +13726,7 @@
 </file>
 
 <file path=xl/drawings/drawing8.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <twoCellAnchor>
     <from>
       <col>4</col>
@@ -13746,9 +13746,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId1"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -13773,9 +13773,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId2"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -13800,9 +13800,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId3"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId3"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -13825,24 +13825,24 @@
       <nvPicPr>
         <cNvPr id="2" name="Imagem 1" descr="logo_red.png"/>
         <cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
+          <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
         </cNvPicPr>
       </nvPicPr>
       <blipFill>
-        <a:blip r:embed="rId4"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId4"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:xfrm>
+        <a:xfrm xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:off x="2189823" y="183077"/>
           <a:ext cx="3726883" cy="786760"/>
         </a:xfrm>
-        <a:prstGeom prst="rect">
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect">
           <avLst/>
         </a:prstGeom>
-        <a:ln>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:prstDash val="solid"/>
         </a:ln>
       </spPr>
@@ -13853,7 +13853,7 @@
 </file>
 
 <file path=xl/drawings/drawing9.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <twoCellAnchor>
     <from>
       <col>3</col>
@@ -13873,9 +13873,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId1"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -15620,7 +15620,7 @@
       </c>
       <c r="E20" s="53" t="inlineStr">
         <is>
-          <t> </t>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
       <c r="F20" s="53" t="n"/>
@@ -16730,7 +16730,7 @@
       </c>
       <c r="E20" s="53" t="inlineStr">
         <is>
-          <t> </t>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
       <c r="F20" s="53" t="n"/>
@@ -18327,7 +18327,7 @@
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t> </t>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
       <c r="Z25" s="154" t="inlineStr">
@@ -20529,7 +20529,7 @@
       <c r="X18" s="24" t="n"/>
       <c r="AN18" t="inlineStr">
         <is>
-          <t> </t>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
     </row>
@@ -21183,7 +21183,7 @@
       <c r="X18" s="24" t="n"/>
       <c r="AN18" t="inlineStr">
         <is>
-          <t> </t>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
     </row>
@@ -21705,7 +21705,7 @@
       <c r="X18" s="24" t="n"/>
       <c r="AN18" t="inlineStr">
         <is>
-          <t> </t>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
     </row>
@@ -22364,7 +22364,7 @@
       <c r="W18" s="24" t="n"/>
       <c r="AM18" t="inlineStr">
         <is>
-          <t> </t>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
     </row>
@@ -22997,7 +22997,7 @@
       </c>
       <c r="AM18" t="inlineStr">
         <is>
-          <t> </t>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
     </row>
@@ -23541,7 +23541,7 @@
         </is>
       </c>
       <c r="B14" s="234" t="n">
-        <v>1100</v>
+        <v>1770</v>
       </c>
       <c r="C14" s="251" t="n">
         <v>100</v>
@@ -23603,7 +23603,7 @@
       </c>
       <c r="AL18" t="inlineStr">
         <is>
-          <t> </t>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
     </row>
@@ -24544,7 +24544,7 @@
       <c r="D20" s="194" t="n"/>
       <c r="E20" s="53" t="inlineStr">
         <is>
-          <t> </t>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
       <c r="F20" s="53" t="n"/>
@@ -26214,7 +26214,7 @@
       <c r="D20" s="194" t="n"/>
       <c r="E20" s="53" t="inlineStr">
         <is>
-          <t> </t>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
       <c r="F20" s="53" t="n"/>
@@ -27136,7 +27136,7 @@
       </c>
       <c r="E20" s="53" t="inlineStr">
         <is>
-          <t> </t>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
       <c r="F20" s="53" t="n"/>
@@ -28084,7 +28084,7 @@
       </c>
       <c r="E20" s="53" t="inlineStr">
         <is>
-          <t> </t>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
       <c r="F20" s="53" t="n"/>
@@ -29066,7 +29066,7 @@
       </c>
       <c r="E20" s="53" t="inlineStr">
         <is>
-          <t> </t>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
       <c r="F20" s="53" t="n"/>
@@ -30024,7 +30024,7 @@
       </c>
       <c r="E20" s="53" t="inlineStr">
         <is>
-          <t> </t>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
       <c r="F20" s="53" t="n"/>
@@ -31088,7 +31088,7 @@
       </c>
       <c r="E20" s="53" t="inlineStr">
         <is>
-          <t> </t>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
       <c r="F20" s="53" t="n"/>
@@ -32102,7 +32102,7 @@
       </c>
       <c r="E20" s="53" t="inlineStr">
         <is>
-          <t> </t>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
       <c r="F20" s="53" t="n"/>

</xml_diff>